<commit_message>
:card_file_box: tabela modulo_selimp + refresh nas importações e leitura no dashboard
</commit_message>
<xml_diff>
--- a/docs/ipt/SETORES.xlsx
+++ b/docs/ipt/SETORES.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcos.silva\Documents\Code\ADC Control\limpebras-flip_control\docs\ipt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2101D332-D607-4DE4-A6CA-C35F9F09F9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA67E153-D05A-4637-AEB0-550EAD9FDE74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="791" xr2:uid="{8E173A8B-8DE5-4C92-9B13-B8B49F4B4ED8}"/>
+    <workbookView xWindow="-20610" yWindow="2775" windowWidth="20730" windowHeight="11040" tabRatio="791" xr2:uid="{8E173A8B-8DE5-4C92-9B13-B8B49F4B4ED8}"/>
   </bookViews>
   <sheets>
     <sheet name="SETORES" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">SETORES!$A$1:$J$287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SETORES!$A$1:$J$402</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">SETORES!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -3231,8 +3231,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="23" x14ac:knownFonts="1">
     <font>
@@ -3824,7 +3825,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3887,6 +3888,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="33" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4394,7 +4407,7 @@
       <c r="G2" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="22">
         <v>45997</v>
       </c>
       <c r="I2" s="9" t="s">
@@ -4426,7 +4439,7 @@
       <c r="G3" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="22">
         <v>45997</v>
       </c>
       <c r="I3" s="9" t="s">
@@ -4458,7 +4471,7 @@
       <c r="G4" s="8" t="s">
         <v>372</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="23">
         <v>45994</v>
       </c>
       <c r="I4" s="9" t="s">
@@ -4490,7 +4503,7 @@
       <c r="G5" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="23">
         <v>45994</v>
       </c>
       <c r="I5" s="9" t="s">
@@ -4522,7 +4535,7 @@
       <c r="G6" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="23">
         <v>45995</v>
       </c>
       <c r="I6" s="9" t="s">
@@ -4554,7 +4567,7 @@
       <c r="G7" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="23">
         <v>45994</v>
       </c>
       <c r="I7" s="9" t="s">
@@ -4586,7 +4599,7 @@
       <c r="G8" s="8" t="s">
         <v>313</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="23">
         <v>45994</v>
       </c>
       <c r="I8" s="9" t="s">
@@ -4618,7 +4631,7 @@
       <c r="G9" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="23">
         <v>45994</v>
       </c>
       <c r="I9" s="9" t="s">
@@ -4650,7 +4663,7 @@
       <c r="G10" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="23">
         <v>45994</v>
       </c>
       <c r="I10" s="9" t="s">
@@ -4682,7 +4695,7 @@
       <c r="G11" s="8" t="s">
         <v>367</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="23">
         <v>45994</v>
       </c>
       <c r="I11" s="9" t="s">
@@ -4714,7 +4727,7 @@
       <c r="G12" s="8" t="s">
         <v>366</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="23">
         <v>45994</v>
       </c>
       <c r="I12" s="9" t="s">
@@ -4746,7 +4759,7 @@
       <c r="G13" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="23">
         <v>45994</v>
       </c>
       <c r="I13" s="9" t="s">
@@ -4778,7 +4791,7 @@
       <c r="G14" s="8" t="s">
         <v>327</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="23">
         <v>45995</v>
       </c>
       <c r="I14" s="9" t="s">
@@ -4810,7 +4823,7 @@
       <c r="G15" s="8" t="s">
         <v>311</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="23">
         <v>45999</v>
       </c>
       <c r="I15" s="9" t="s">
@@ -4842,7 +4855,7 @@
       <c r="G16" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="23">
         <v>45999</v>
       </c>
       <c r="I16" s="9" t="s">
@@ -4874,7 +4887,7 @@
       <c r="G17" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="23">
         <v>45995</v>
       </c>
       <c r="I17" s="9" t="s">
@@ -4906,7 +4919,7 @@
       <c r="G18" s="8" t="s">
         <v>323</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="23">
         <v>45995</v>
       </c>
       <c r="I18" s="9" t="s">
@@ -4938,7 +4951,7 @@
       <c r="G19" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="23">
         <v>45999</v>
       </c>
       <c r="I19" s="9" t="s">
@@ -4970,7 +4983,7 @@
       <c r="G20" s="8" t="s">
         <v>337</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="23">
         <v>46003</v>
       </c>
       <c r="I20" s="9" t="s">
@@ -5002,7 +5015,7 @@
       <c r="G21" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="23">
         <v>45996</v>
       </c>
       <c r="I21" s="9" t="s">
@@ -5034,7 +5047,7 @@
       <c r="G22" s="8" t="s">
         <v>347</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="23">
         <v>45996</v>
       </c>
       <c r="I22" s="9" t="s">
@@ -5066,7 +5079,7 @@
       <c r="G23" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="23">
         <v>45996</v>
       </c>
       <c r="I23" s="9" t="s">
@@ -5098,7 +5111,7 @@
       <c r="G24" s="8" t="s">
         <v>344</v>
       </c>
-      <c r="H24" s="4">
+      <c r="H24" s="22">
         <v>46007</v>
       </c>
       <c r="I24" s="9" t="s">
@@ -5130,7 +5143,7 @@
       <c r="G25" s="8" t="s">
         <v>336</v>
       </c>
-      <c r="H25" s="4">
+      <c r="H25" s="22">
         <v>46007</v>
       </c>
       <c r="I25" s="9" t="s">
@@ -5162,7 +5175,7 @@
       <c r="G26" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="H26" s="4">
+      <c r="H26" s="22">
         <v>45994</v>
       </c>
       <c r="I26" s="9" t="s">
@@ -5194,7 +5207,7 @@
       <c r="G27" s="8" t="s">
         <v>319</v>
       </c>
-      <c r="H27" s="4">
+      <c r="H27" s="22">
         <v>46008</v>
       </c>
       <c r="I27" s="9" t="s">
@@ -5226,7 +5239,7 @@
       <c r="G28" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="H28" s="4">
+      <c r="H28" s="22">
         <v>45994</v>
       </c>
       <c r="I28" s="9" t="s">
@@ -5258,7 +5271,7 @@
       <c r="G29" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="H29" s="4">
+      <c r="H29" s="22">
         <v>45997</v>
       </c>
       <c r="I29" s="9" t="s">
@@ -5290,7 +5303,7 @@
       <c r="G30" s="8" t="s">
         <v>374</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="23">
         <v>45994</v>
       </c>
       <c r="I30" s="9" t="s">
@@ -5322,7 +5335,7 @@
       <c r="G31" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="23">
         <v>46008</v>
       </c>
       <c r="I31" s="9" t="s">
@@ -5354,7 +5367,7 @@
       <c r="G32" s="8" t="s">
         <v>315</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="23">
         <v>45996</v>
       </c>
       <c r="I32" s="9" t="s">
@@ -5386,7 +5399,7 @@
       <c r="G33" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="23">
         <v>45996</v>
       </c>
       <c r="I33" s="9" t="s">
@@ -5418,7 +5431,7 @@
       <c r="G34" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="23">
         <v>45996</v>
       </c>
       <c r="I34" s="9" t="s">
@@ -5450,7 +5463,7 @@
       <c r="G35" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="23">
         <v>45996</v>
       </c>
       <c r="I35" s="9" t="s">
@@ -5482,7 +5495,7 @@
       <c r="G36" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="23">
         <v>45999</v>
       </c>
       <c r="I36" s="9" t="s">
@@ -5514,7 +5527,7 @@
       <c r="G37" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="23">
         <v>45996</v>
       </c>
       <c r="I37" s="9" t="s">
@@ -5546,7 +5559,7 @@
       <c r="G38" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="H38" s="5">
+      <c r="H38" s="23">
         <v>45999</v>
       </c>
       <c r="I38" s="9" t="s">
@@ -5578,7 +5591,7 @@
       <c r="G39" s="8" t="s">
         <v>358</v>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="23">
         <v>45999</v>
       </c>
       <c r="I39" s="9" t="s">
@@ -5611,7 +5624,7 @@
       <c r="G40" s="8" t="s">
         <v>359</v>
       </c>
-      <c r="H40" s="5">
+      <c r="H40" s="23">
         <v>45999</v>
       </c>
       <c r="I40" s="9" t="s">
@@ -5643,7 +5656,7 @@
       <c r="G41" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="23">
         <v>45996</v>
       </c>
       <c r="I41" s="9" t="s">
@@ -5675,7 +5688,7 @@
       <c r="G42" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="23">
         <v>45999</v>
       </c>
       <c r="I42" s="9" t="s">
@@ -5707,7 +5720,7 @@
       <c r="G43" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="H43" s="5">
+      <c r="H43" s="23">
         <v>45999</v>
       </c>
       <c r="I43" s="9" t="s">
@@ -5739,7 +5752,7 @@
       <c r="G44" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="H44" s="5">
+      <c r="H44" s="23">
         <v>45999</v>
       </c>
       <c r="I44" s="9" t="s">
@@ -5771,7 +5784,7 @@
       <c r="G45" s="8" t="s">
         <v>325</v>
       </c>
-      <c r="H45" s="5">
+      <c r="H45" s="23">
         <v>45999</v>
       </c>
       <c r="I45" s="9" t="s">
@@ -5803,7 +5816,7 @@
       <c r="G46" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="H46" s="5">
+      <c r="H46" s="23">
         <v>45999</v>
       </c>
       <c r="I46" s="9" t="s">
@@ -5835,7 +5848,7 @@
       <c r="G47" s="8" t="s">
         <v>355</v>
       </c>
-      <c r="H47" s="5">
+      <c r="H47" s="23">
         <v>45999</v>
       </c>
       <c r="I47" s="9" t="s">
@@ -5867,7 +5880,7 @@
       <c r="G48" s="8" t="s">
         <v>364</v>
       </c>
-      <c r="H48" s="5">
+      <c r="H48" s="23">
         <v>45996</v>
       </c>
       <c r="I48" s="9" t="s">
@@ -5899,7 +5912,7 @@
       <c r="G49" s="8" t="s">
         <v>324</v>
       </c>
-      <c r="H49" s="5">
+      <c r="H49" s="23">
         <v>45996</v>
       </c>
       <c r="I49" s="9" t="s">
@@ -5931,7 +5944,7 @@
       <c r="G50" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="H50" s="5">
+      <c r="H50" s="23">
         <v>45993</v>
       </c>
       <c r="I50" s="9" t="s">
@@ -5963,7 +5976,7 @@
       <c r="G51" s="8" t="s">
         <v>328</v>
       </c>
-      <c r="H51" s="5">
+      <c r="H51" s="23">
         <v>45995</v>
       </c>
       <c r="I51" s="9" t="s">
@@ -5995,7 +6008,7 @@
       <c r="G52" s="8" t="s">
         <v>329</v>
       </c>
-      <c r="H52" s="5">
+      <c r="H52" s="23">
         <v>45995</v>
       </c>
       <c r="I52" s="9" t="s">
@@ -6027,7 +6040,7 @@
       <c r="G53" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="H53" s="5">
+      <c r="H53" s="23">
         <v>45995</v>
       </c>
       <c r="I53" s="9" t="s">
@@ -6059,7 +6072,7 @@
       <c r="G54" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="H54" s="5">
+      <c r="H54" s="23">
         <v>45993</v>
       </c>
       <c r="I54" s="9" t="s">
@@ -6091,7 +6104,7 @@
       <c r="G55" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="H55" s="5">
+      <c r="H55" s="23">
         <v>45993</v>
       </c>
       <c r="I55" s="9" t="s">
@@ -6123,7 +6136,7 @@
       <c r="G56" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="H56" s="5">
+      <c r="H56" s="23">
         <v>45993</v>
       </c>
       <c r="I56" s="9" t="s">
@@ -6155,7 +6168,7 @@
       <c r="G57" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="H57" s="5">
+      <c r="H57" s="23">
         <v>45995</v>
       </c>
       <c r="I57" s="9" t="s">
@@ -6187,7 +6200,7 @@
       <c r="G58" s="8" t="s">
         <v>299</v>
       </c>
-      <c r="H58" s="5">
+      <c r="H58" s="23">
         <v>45993</v>
       </c>
       <c r="I58" s="9" t="s">
@@ -6219,7 +6232,7 @@
       <c r="G59" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="H59" s="5">
+      <c r="H59" s="23">
         <v>45993</v>
       </c>
       <c r="I59" s="9" t="s">
@@ -6251,7 +6264,7 @@
       <c r="G60" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="H60" s="5">
+      <c r="H60" s="23">
         <v>45993</v>
       </c>
       <c r="I60" s="9" t="s">
@@ -6283,7 +6296,7 @@
       <c r="G61" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="H61" s="5">
+      <c r="H61" s="23">
         <v>45993</v>
       </c>
       <c r="I61" s="9" t="s">
@@ -6315,7 +6328,7 @@
       <c r="G62" s="8" t="s">
         <v>303</v>
       </c>
-      <c r="H62" s="5">
+      <c r="H62" s="23">
         <v>45993</v>
       </c>
       <c r="I62" s="9" t="s">
@@ -6347,7 +6360,7 @@
       <c r="G63" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="H63" s="5">
+      <c r="H63" s="23">
         <v>45995</v>
       </c>
       <c r="I63" s="9" t="s">
@@ -6379,7 +6392,7 @@
       <c r="G64" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="H64" s="5">
+      <c r="H64" s="23">
         <v>45993</v>
       </c>
       <c r="I64" s="9" t="s">
@@ -6411,7 +6424,7 @@
       <c r="G65" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="H65" s="5">
+      <c r="H65" s="23">
         <v>45995</v>
       </c>
       <c r="I65" s="9" t="s">
@@ -6443,7 +6456,7 @@
       <c r="G66" s="8" t="s">
         <v>333</v>
       </c>
-      <c r="H66" s="5">
+      <c r="H66" s="23">
         <v>45995</v>
       </c>
       <c r="I66" s="9" t="s">
@@ -6475,7 +6488,7 @@
       <c r="G67" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="H67" s="5">
+      <c r="H67" s="23">
         <v>45995</v>
       </c>
       <c r="I67" s="9" t="s">
@@ -6507,7 +6520,7 @@
       <c r="G68" s="6" t="s">
         <v>936</v>
       </c>
-      <c r="H68" s="5">
+      <c r="H68" s="23">
         <v>46105</v>
       </c>
       <c r="I68" s="9" t="s">
@@ -6539,7 +6552,7 @@
       <c r="G69" s="6" t="s">
         <v>771</v>
       </c>
-      <c r="H69" s="5">
+      <c r="H69" s="23">
         <v>46105</v>
       </c>
       <c r="I69" s="9" t="s">
@@ -6571,7 +6584,7 @@
       <c r="G70" s="6" t="s">
         <v>753</v>
       </c>
-      <c r="H70" s="5">
+      <c r="H70" s="23">
         <v>46105</v>
       </c>
       <c r="I70" s="9" t="s">
@@ -6603,7 +6616,7 @@
       <c r="G71" s="6" t="s">
         <v>819</v>
       </c>
-      <c r="H71" s="5">
+      <c r="H71" s="23">
         <v>46105</v>
       </c>
       <c r="I71" s="9" t="s">
@@ -6635,7 +6648,7 @@
       <c r="G72" s="6" t="s">
         <v>770</v>
       </c>
-      <c r="H72" s="5">
+      <c r="H72" s="23">
         <v>46101</v>
       </c>
       <c r="I72" s="9" t="s">
@@ -6667,7 +6680,7 @@
       <c r="G73" s="6" t="s">
         <v>765</v>
       </c>
-      <c r="H73" s="5">
+      <c r="H73" s="23">
         <v>46101</v>
       </c>
       <c r="I73" s="9" t="s">
@@ -6699,7 +6712,7 @@
       <c r="G74" s="6" t="s">
         <v>764</v>
       </c>
-      <c r="H74" s="5">
+      <c r="H74" s="23">
         <v>46101</v>
       </c>
       <c r="I74" s="9" t="s">
@@ -6731,7 +6744,7 @@
       <c r="G75" s="6" t="s">
         <v>772</v>
       </c>
-      <c r="H75" s="5">
+      <c r="H75" s="23">
         <v>46101</v>
       </c>
       <c r="I75" s="9" t="s">
@@ -6763,7 +6776,7 @@
       <c r="G76" s="6" t="s">
         <v>769</v>
       </c>
-      <c r="H76" s="5">
+      <c r="H76" s="23">
         <v>46101</v>
       </c>
       <c r="I76" s="9" t="s">
@@ -6795,7 +6808,7 @@
       <c r="G77" s="6" t="s">
         <v>774</v>
       </c>
-      <c r="H77" s="5">
+      <c r="H77" s="23">
         <v>46101</v>
       </c>
       <c r="I77" s="9" t="s">
@@ -6827,7 +6840,7 @@
       <c r="G78" s="6" t="s">
         <v>763</v>
       </c>
-      <c r="H78" s="5">
+      <c r="H78" s="23">
         <v>46101</v>
       </c>
       <c r="I78" s="9" t="s">
@@ -6859,7 +6872,7 @@
       <c r="G79" s="6" t="s">
         <v>768</v>
       </c>
-      <c r="H79" s="5">
+      <c r="H79" s="23">
         <v>46101</v>
       </c>
       <c r="I79" s="9" t="s">
@@ -6891,7 +6904,7 @@
       <c r="G80" s="6" t="s">
         <v>767</v>
       </c>
-      <c r="H80" s="5">
+      <c r="H80" s="23">
         <v>46101</v>
       </c>
       <c r="I80" s="9" t="s">
@@ -6923,7 +6936,7 @@
       <c r="G81" s="6" t="s">
         <v>761</v>
       </c>
-      <c r="H81" s="5">
+      <c r="H81" s="23">
         <v>46101</v>
       </c>
       <c r="I81" s="9" t="s">
@@ -6955,7 +6968,7 @@
       <c r="G82" s="6" t="s">
         <v>773</v>
       </c>
-      <c r="H82" s="5">
+      <c r="H82" s="23">
         <v>46101</v>
       </c>
       <c r="I82" s="9" t="s">
@@ -6987,7 +7000,7 @@
       <c r="G83" s="6" t="s">
         <v>766</v>
       </c>
-      <c r="H83" s="5">
+      <c r="H83" s="23">
         <v>46102</v>
       </c>
       <c r="I83" s="9" t="s">
@@ -7019,7 +7032,7 @@
       <c r="G84" s="6" t="s">
         <v>762</v>
       </c>
-      <c r="H84" s="5">
+      <c r="H84" s="23">
         <v>46101</v>
       </c>
       <c r="I84" s="9" t="s">
@@ -7051,7 +7064,7 @@
       <c r="G85" s="6" t="s">
         <v>760</v>
       </c>
-      <c r="H85" s="5">
+      <c r="H85" s="23">
         <v>46102</v>
       </c>
       <c r="I85" s="9" t="s">
@@ -7083,7 +7096,7 @@
       <c r="G86" s="6" t="s">
         <v>756</v>
       </c>
-      <c r="H86" s="5">
+      <c r="H86" s="23">
         <v>46101</v>
       </c>
       <c r="I86" s="9" t="s">
@@ -7115,7 +7128,7 @@
       <c r="G87" s="6" t="s">
         <v>757</v>
       </c>
-      <c r="H87" s="5">
+      <c r="H87" s="23">
         <v>46101</v>
       </c>
       <c r="I87" s="9" t="s">
@@ -7147,7 +7160,7 @@
       <c r="G88" s="6" t="s">
         <v>752</v>
       </c>
-      <c r="H88" s="5">
+      <c r="H88" s="23">
         <v>46101</v>
       </c>
       <c r="I88" s="9" t="s">
@@ -7179,7 +7192,7 @@
       <c r="G89" s="6" t="s">
         <v>759</v>
       </c>
-      <c r="H89" s="5">
+      <c r="H89" s="23">
         <v>46101</v>
       </c>
       <c r="I89" s="9" t="s">
@@ -7211,7 +7224,7 @@
       <c r="G90" s="6" t="s">
         <v>758</v>
       </c>
-      <c r="H90" s="5">
+      <c r="H90" s="23">
         <v>46101</v>
       </c>
       <c r="I90" s="9" t="s">
@@ -7243,7 +7256,7 @@
       <c r="G91" s="6" t="s">
         <v>754</v>
       </c>
-      <c r="H91" s="5">
+      <c r="H91" s="23">
         <v>46101</v>
       </c>
       <c r="I91" s="9" t="s">
@@ -7275,7 +7288,7 @@
       <c r="G92" s="6" t="s">
         <v>755</v>
       </c>
-      <c r="H92" s="5">
+      <c r="H92" s="23">
         <v>46101</v>
       </c>
       <c r="I92" s="9" t="s">
@@ -7307,7 +7320,7 @@
       <c r="G93" s="6" t="s">
         <v>751</v>
       </c>
-      <c r="H93" s="5">
+      <c r="H93" s="23">
         <v>46101</v>
       </c>
       <c r="I93" s="9" t="s">
@@ -7339,7 +7352,7 @@
       <c r="G94" s="6" t="s">
         <v>818</v>
       </c>
-      <c r="H94" s="5">
+      <c r="H94" s="23">
         <v>46101</v>
       </c>
       <c r="I94" s="9" t="s">
@@ -7371,7 +7384,7 @@
       <c r="G95" s="6" t="s">
         <v>807</v>
       </c>
-      <c r="H95" s="5">
+      <c r="H95" s="23">
         <v>46104</v>
       </c>
       <c r="I95" s="9" t="s">
@@ -7403,7 +7416,7 @@
       <c r="G96" s="6" t="s">
         <v>805</v>
       </c>
-      <c r="H96" s="5">
+      <c r="H96" s="23">
         <v>46104</v>
       </c>
       <c r="I96" s="9" t="s">
@@ -7435,7 +7448,7 @@
       <c r="G97" s="6" t="s">
         <v>816</v>
       </c>
-      <c r="H97" s="5">
+      <c r="H97" s="23">
         <v>46104</v>
       </c>
       <c r="I97" s="9" t="s">
@@ -7467,7 +7480,7 @@
       <c r="G98" s="6" t="s">
         <v>815</v>
       </c>
-      <c r="H98" s="5">
+      <c r="H98" s="23">
         <v>46104</v>
       </c>
       <c r="I98" s="9" t="s">
@@ -7499,7 +7512,7 @@
       <c r="G99" s="6" t="s">
         <v>813</v>
       </c>
-      <c r="H99" s="5">
+      <c r="H99" s="23">
         <v>46104</v>
       </c>
       <c r="I99" s="9" t="s">
@@ -7531,7 +7544,7 @@
       <c r="G100" s="6" t="s">
         <v>814</v>
       </c>
-      <c r="H100" s="5">
+      <c r="H100" s="23">
         <v>46104</v>
       </c>
       <c r="I100" s="9" t="s">
@@ -7563,7 +7576,7 @@
       <c r="G101" s="6" t="s">
         <v>784</v>
       </c>
-      <c r="H101" s="5">
+      <c r="H101" s="23">
         <v>46104</v>
       </c>
       <c r="I101" s="9" t="s">
@@ -7595,7 +7608,7 @@
       <c r="G102" s="6" t="s">
         <v>797</v>
       </c>
-      <c r="H102" s="5">
+      <c r="H102" s="23">
         <v>46104</v>
       </c>
       <c r="I102" s="9" t="s">
@@ -7627,7 +7640,7 @@
       <c r="G103" s="6" t="s">
         <v>808</v>
       </c>
-      <c r="H103" s="5">
+      <c r="H103" s="23">
         <v>46104</v>
       </c>
       <c r="I103" s="9" t="s">
@@ -7659,7 +7672,7 @@
       <c r="G104" s="6" t="s">
         <v>792</v>
       </c>
-      <c r="H104" s="5">
+      <c r="H104" s="23">
         <v>46104</v>
       </c>
       <c r="I104" s="9" t="s">
@@ -7691,7 +7704,7 @@
       <c r="G105" s="6" t="s">
         <v>798</v>
       </c>
-      <c r="H105" s="5">
+      <c r="H105" s="23">
         <v>46104</v>
       </c>
       <c r="I105" s="9" t="s">
@@ -7723,7 +7736,7 @@
       <c r="G106" s="6" t="s">
         <v>817</v>
       </c>
-      <c r="H106" s="5">
+      <c r="H106" s="23">
         <v>46104</v>
       </c>
       <c r="I106" s="9" t="s">
@@ -7755,7 +7768,7 @@
       <c r="G107" s="6" t="s">
         <v>810</v>
       </c>
-      <c r="H107" s="5">
+      <c r="H107" s="23">
         <v>46104</v>
       </c>
       <c r="I107" s="9" t="s">
@@ -7787,7 +7800,7 @@
       <c r="G108" s="6" t="s">
         <v>802</v>
       </c>
-      <c r="H108" s="5">
+      <c r="H108" s="23">
         <v>46104</v>
       </c>
       <c r="I108" s="9" t="s">
@@ -7819,7 +7832,7 @@
       <c r="G109" s="6" t="s">
         <v>795</v>
       </c>
-      <c r="H109" s="5">
+      <c r="H109" s="23">
         <v>46104</v>
       </c>
       <c r="I109" s="9" t="s">
@@ -7851,7 +7864,7 @@
       <c r="G110" s="6" t="s">
         <v>786</v>
       </c>
-      <c r="H110" s="5">
+      <c r="H110" s="23">
         <v>46105</v>
       </c>
       <c r="I110" s="9" t="s">
@@ -7883,7 +7896,7 @@
       <c r="G111" s="6" t="s">
         <v>778</v>
       </c>
-      <c r="H111" s="5">
+      <c r="H111" s="23">
         <v>46105</v>
       </c>
       <c r="I111" s="9" t="s">
@@ -7915,7 +7928,7 @@
       <c r="G112" s="6" t="s">
         <v>804</v>
       </c>
-      <c r="H112" s="5">
+      <c r="H112" s="23">
         <v>46105</v>
       </c>
       <c r="I112" s="9" t="s">
@@ -7947,7 +7960,7 @@
       <c r="G113" s="6" t="s">
         <v>811</v>
       </c>
-      <c r="H113" s="5">
+      <c r="H113" s="23">
         <v>46105</v>
       </c>
       <c r="I113" s="9" t="s">
@@ -7979,7 +7992,7 @@
       <c r="G114" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="H114" s="5">
+      <c r="H114" s="23">
         <v>46105</v>
       </c>
       <c r="I114" s="9" t="s">
@@ -8011,7 +8024,7 @@
       <c r="G115" s="6" t="s">
         <v>794</v>
       </c>
-      <c r="H115" s="5">
+      <c r="H115" s="23">
         <v>46105</v>
       </c>
       <c r="I115" s="9" t="s">
@@ -8043,7 +8056,7 @@
       <c r="G116" s="6" t="s">
         <v>777</v>
       </c>
-      <c r="H116" s="5">
+      <c r="H116" s="23">
         <v>46105</v>
       </c>
       <c r="I116" s="9" t="s">
@@ -8075,7 +8088,7 @@
       <c r="G117" s="6" t="s">
         <v>788</v>
       </c>
-      <c r="H117" s="5">
+      <c r="H117" s="23">
         <v>46105</v>
       </c>
       <c r="I117" s="9" t="s">
@@ -8107,7 +8120,7 @@
       <c r="G118" s="6" t="s">
         <v>776</v>
       </c>
-      <c r="H118" s="5">
+      <c r="H118" s="23">
         <v>46105</v>
       </c>
       <c r="I118" s="9" t="s">
@@ -8139,7 +8152,7 @@
       <c r="G119" s="6" t="s">
         <v>782</v>
       </c>
-      <c r="H119" s="5">
+      <c r="H119" s="23">
         <v>46105</v>
       </c>
       <c r="I119" s="9" t="s">
@@ -8171,7 +8184,7 @@
       <c r="G120" s="6" t="s">
         <v>806</v>
       </c>
-      <c r="H120" s="5">
+      <c r="H120" s="23">
         <v>46105</v>
       </c>
       <c r="I120" s="9" t="s">
@@ -8203,7 +8216,7 @@
       <c r="G121" s="6" t="s">
         <v>787</v>
       </c>
-      <c r="H121" s="5">
+      <c r="H121" s="23">
         <v>46105</v>
       </c>
       <c r="I121" s="9" t="s">
@@ -8235,7 +8248,7 @@
       <c r="G122" s="6" t="s">
         <v>793</v>
       </c>
-      <c r="H122" s="5">
+      <c r="H122" s="23">
         <v>46105</v>
       </c>
       <c r="I122" s="9" t="s">
@@ -8267,7 +8280,7 @@
       <c r="G123" s="6" t="s">
         <v>800</v>
       </c>
-      <c r="H123" s="5">
+      <c r="H123" s="23">
         <v>46105</v>
       </c>
       <c r="I123" s="9" t="s">
@@ -8299,7 +8312,7 @@
       <c r="G124" s="6" t="s">
         <v>812</v>
       </c>
-      <c r="H124" s="5">
+      <c r="H124" s="23">
         <v>46105</v>
       </c>
       <c r="I124" s="9" t="s">
@@ -8331,7 +8344,7 @@
       <c r="G125" s="6" t="s">
         <v>824</v>
       </c>
-      <c r="H125" s="5">
+      <c r="H125" s="23">
         <v>46102</v>
       </c>
       <c r="I125" s="9" t="s">
@@ -8363,7 +8376,7 @@
       <c r="G126" s="6" t="s">
         <v>821</v>
       </c>
-      <c r="H126" s="5">
+      <c r="H126" s="23">
         <v>46102</v>
       </c>
       <c r="I126" s="9" t="s">
@@ -8395,7 +8408,7 @@
       <c r="G127" s="6" t="s">
         <v>822</v>
       </c>
-      <c r="H127" s="5">
+      <c r="H127" s="23">
         <v>46102</v>
       </c>
       <c r="I127" s="9" t="s">
@@ -8427,7 +8440,7 @@
       <c r="G128" s="6" t="s">
         <v>825</v>
       </c>
-      <c r="H128" s="5">
+      <c r="H128" s="23">
         <v>46102</v>
       </c>
       <c r="I128" s="9" t="s">
@@ -8459,7 +8472,7 @@
       <c r="G129" s="6" t="s">
         <v>831</v>
       </c>
-      <c r="H129" s="5">
+      <c r="H129" s="23">
         <v>46102</v>
       </c>
       <c r="I129" s="9" t="s">
@@ -8491,7 +8504,7 @@
       <c r="G130" s="6" t="s">
         <v>820</v>
       </c>
-      <c r="H130" s="5">
+      <c r="H130" s="23">
         <v>46102</v>
       </c>
       <c r="I130" s="9" t="s">
@@ -8523,7 +8536,7 @@
       <c r="G131" s="6" t="s">
         <v>823</v>
       </c>
-      <c r="H131" s="5">
+      <c r="H131" s="23">
         <v>46105</v>
       </c>
       <c r="I131" s="9" t="s">
@@ -8555,7 +8568,7 @@
       <c r="G132" s="6" t="s">
         <v>833</v>
       </c>
-      <c r="H132" s="5">
+      <c r="H132" s="23">
         <v>46102</v>
       </c>
       <c r="I132" s="9" t="s">
@@ -8587,7 +8600,7 @@
       <c r="G133" s="6" t="s">
         <v>826</v>
       </c>
-      <c r="H133" s="5">
+      <c r="H133" s="23">
         <v>46106</v>
       </c>
       <c r="I133" s="9" t="s">
@@ -8619,7 +8632,7 @@
       <c r="G134" s="6" t="s">
         <v>834</v>
       </c>
-      <c r="H134" s="5">
+      <c r="H134" s="23">
         <v>46102</v>
       </c>
       <c r="I134" s="9" t="s">
@@ -8651,7 +8664,7 @@
       <c r="G135" s="6" t="s">
         <v>832</v>
       </c>
-      <c r="H135" s="5">
+      <c r="H135" s="23">
         <v>46102</v>
       </c>
       <c r="I135" s="9" t="s">
@@ -8683,7 +8696,7 @@
       <c r="G136" s="6" t="s">
         <v>827</v>
       </c>
-      <c r="H136" s="5">
+      <c r="H136" s="23">
         <v>46102</v>
       </c>
       <c r="I136" s="9" t="s">
@@ -8715,7 +8728,7 @@
       <c r="G137" s="6" t="s">
         <v>828</v>
       </c>
-      <c r="H137" s="5">
+      <c r="H137" s="23">
         <v>46102</v>
       </c>
       <c r="I137" s="9" t="s">
@@ -8747,7 +8760,7 @@
       <c r="G138" s="6" t="s">
         <v>829</v>
       </c>
-      <c r="H138" s="5">
+      <c r="H138" s="23">
         <v>46102</v>
       </c>
       <c r="I138" s="9" t="s">
@@ -8779,7 +8792,7 @@
       <c r="G139" s="6" t="s">
         <v>830</v>
       </c>
-      <c r="H139" s="5">
+      <c r="H139" s="23">
         <v>46102</v>
       </c>
       <c r="I139" s="9" t="s">
@@ -8811,7 +8824,7 @@
       <c r="G140" s="6" t="s">
         <v>779</v>
       </c>
-      <c r="H140" s="5">
+      <c r="H140" s="23">
         <v>46104</v>
       </c>
       <c r="I140" s="9" t="s">
@@ -8843,7 +8856,7 @@
       <c r="G141" s="6" t="s">
         <v>780</v>
       </c>
-      <c r="H141" s="5">
+      <c r="H141" s="23">
         <v>46104</v>
       </c>
       <c r="I141" s="9" t="s">
@@ -8875,7 +8888,7 @@
       <c r="G142" s="6" t="s">
         <v>785</v>
       </c>
-      <c r="H142" s="5">
+      <c r="H142" s="23">
         <v>46104</v>
       </c>
       <c r="I142" s="9" t="s">
@@ -8907,7 +8920,7 @@
       <c r="G143" s="6" t="s">
         <v>781</v>
       </c>
-      <c r="H143" s="5">
+      <c r="H143" s="23">
         <v>46104</v>
       </c>
       <c r="I143" s="9" t="s">
@@ -8939,7 +8952,7 @@
       <c r="G144" s="6" t="s">
         <v>789</v>
       </c>
-      <c r="H144" s="5">
+      <c r="H144" s="23">
         <v>46104</v>
       </c>
       <c r="I144" s="9" t="s">
@@ -8971,7 +8984,7 @@
       <c r="G145" s="6" t="s">
         <v>809</v>
       </c>
-      <c r="H145" s="5">
+      <c r="H145" s="23">
         <v>46104</v>
       </c>
       <c r="I145" s="9" t="s">
@@ -9003,7 +9016,7 @@
       <c r="G146" s="6" t="s">
         <v>799</v>
       </c>
-      <c r="H146" s="5">
+      <c r="H146" s="23">
         <v>46102</v>
       </c>
       <c r="I146" s="9" t="s">
@@ -9035,7 +9048,7 @@
       <c r="G147" s="6" t="s">
         <v>791</v>
       </c>
-      <c r="H147" s="5">
+      <c r="H147" s="23">
         <v>46102</v>
       </c>
       <c r="I147" s="9" t="s">
@@ -9067,7 +9080,7 @@
       <c r="G148" s="6" t="s">
         <v>790</v>
       </c>
-      <c r="H148" s="5">
+      <c r="H148" s="23">
         <v>46102</v>
       </c>
       <c r="I148" s="9" t="s">
@@ -9099,7 +9112,7 @@
       <c r="G149" s="6" t="s">
         <v>796</v>
       </c>
-      <c r="H149" s="5">
+      <c r="H149" s="23">
         <v>46102</v>
       </c>
       <c r="I149" s="9" t="s">
@@ -9131,7 +9144,7 @@
       <c r="G150" s="6" t="s">
         <v>783</v>
       </c>
-      <c r="H150" s="5">
+      <c r="H150" s="23">
         <v>46102</v>
       </c>
       <c r="I150" s="9" t="s">
@@ -9163,7 +9176,7 @@
       <c r="G151" s="6" t="s">
         <v>803</v>
       </c>
-      <c r="H151" s="5">
+      <c r="H151" s="23">
         <v>46102</v>
       </c>
       <c r="I151" s="9" t="s">
@@ -9195,7 +9208,7 @@
       <c r="G152" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="H152" s="4">
+      <c r="H152" s="22">
         <v>46006</v>
       </c>
       <c r="I152" s="9">
@@ -9227,7 +9240,7 @@
       <c r="G153" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="H153" s="4">
+      <c r="H153" s="22">
         <v>46006</v>
       </c>
       <c r="I153" s="9">
@@ -9259,7 +9272,7 @@
       <c r="G154" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="H154" s="4">
+      <c r="H154" s="22">
         <v>46006</v>
       </c>
       <c r="I154" s="9">
@@ -9291,7 +9304,7 @@
       <c r="G155" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="H155" s="4">
+      <c r="H155" s="22">
         <v>46007</v>
       </c>
       <c r="I155" s="9">
@@ -9323,7 +9336,7 @@
       <c r="G156" s="6" t="s">
         <v>379</v>
       </c>
-      <c r="H156" s="4">
+      <c r="H156" s="22">
         <v>46006</v>
       </c>
       <c r="I156" s="9">
@@ -9355,7 +9368,7 @@
       <c r="G157" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="H157" s="4">
+      <c r="H157" s="22">
         <v>46007</v>
       </c>
       <c r="I157" s="9">
@@ -9387,7 +9400,7 @@
       <c r="G158" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="H158" s="4">
+      <c r="H158" s="22">
         <v>46006</v>
       </c>
       <c r="I158" s="9" t="s">
@@ -9419,7 +9432,7 @@
       <c r="G159" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="H159" s="4">
+      <c r="H159" s="22">
         <v>46007</v>
       </c>
       <c r="I159" s="9">
@@ -9451,7 +9464,7 @@
       <c r="G160" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="H160" s="4">
+      <c r="H160" s="22">
         <v>46006</v>
       </c>
       <c r="I160" s="9">
@@ -9483,7 +9496,7 @@
       <c r="G161" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="H161" s="4">
+      <c r="H161" s="22">
         <v>46007</v>
       </c>
       <c r="I161" s="9">
@@ -9515,7 +9528,7 @@
       <c r="G162" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="H162" s="4">
+      <c r="H162" s="22">
         <v>46006</v>
       </c>
       <c r="I162" s="9">
@@ -9547,7 +9560,7 @@
       <c r="G163" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="H163" s="4">
+      <c r="H163" s="22">
         <v>46000</v>
       </c>
       <c r="I163" s="9">
@@ -9579,7 +9592,7 @@
       <c r="G164" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="H164" s="4">
+      <c r="H164" s="22">
         <v>46003</v>
       </c>
       <c r="I164" s="9">
@@ -9611,7 +9624,7 @@
       <c r="G165" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="H165" s="4">
+      <c r="H165" s="22">
         <v>46002</v>
       </c>
       <c r="I165" s="9">
@@ -9643,7 +9656,7 @@
       <c r="G166" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="H166" s="4">
+      <c r="H166" s="22">
         <v>46006</v>
       </c>
       <c r="I166" s="9">
@@ -9675,7 +9688,7 @@
       <c r="G167" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="H167" s="4">
+      <c r="H167" s="22">
         <v>46002</v>
       </c>
       <c r="I167" s="9">
@@ -9707,7 +9720,7 @@
       <c r="G168" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="H168" s="4">
+      <c r="H168" s="22">
         <v>46002</v>
       </c>
       <c r="I168" s="9">
@@ -9739,7 +9752,7 @@
       <c r="G169" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="H169" s="4">
+      <c r="H169" s="22">
         <v>46002</v>
       </c>
       <c r="I169" s="9" t="s">
@@ -9771,7 +9784,7 @@
       <c r="G170" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="H170" s="4">
+      <c r="H170" s="22">
         <v>46002</v>
       </c>
       <c r="I170" s="9" t="s">
@@ -9803,7 +9816,7 @@
       <c r="G171" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="H171" s="4">
+      <c r="H171" s="22">
         <v>46002</v>
       </c>
       <c r="I171" s="9" t="s">
@@ -9835,7 +9848,7 @@
       <c r="G172" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="H172" s="4">
+      <c r="H172" s="22">
         <v>46002</v>
       </c>
       <c r="I172" s="9">
@@ -9867,7 +9880,7 @@
       <c r="G173" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="H173" s="4">
+      <c r="H173" s="22">
         <v>46002</v>
       </c>
       <c r="I173" s="9">
@@ -9899,7 +9912,7 @@
       <c r="G174" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="H174" s="4">
+      <c r="H174" s="22">
         <v>46002</v>
       </c>
       <c r="I174" s="9">
@@ -9931,7 +9944,7 @@
       <c r="G175" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="H175" s="4">
+      <c r="H175" s="22">
         <v>46002</v>
       </c>
       <c r="I175" s="9">
@@ -9963,7 +9976,7 @@
       <c r="G176" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="H176" s="4">
+      <c r="H176" s="22">
         <v>46002</v>
       </c>
       <c r="I176" s="9">
@@ -9995,7 +10008,7 @@
       <c r="G177" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="H177" s="4">
+      <c r="H177" s="22">
         <v>46002</v>
       </c>
       <c r="I177" s="9">
@@ -10027,7 +10040,7 @@
       <c r="G178" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H178" s="4">
+      <c r="H178" s="22">
         <v>46002</v>
       </c>
       <c r="I178" s="9">
@@ -10059,7 +10072,7 @@
       <c r="G179" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="H179" s="4">
+      <c r="H179" s="22">
         <v>46002</v>
       </c>
       <c r="I179" s="9">
@@ -10091,7 +10104,7 @@
       <c r="G180" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="H180" s="4">
+      <c r="H180" s="22">
         <v>46006</v>
       </c>
       <c r="I180" s="9">
@@ -10123,7 +10136,7 @@
       <c r="G181" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="H181" s="4">
+      <c r="H181" s="22">
         <v>46002</v>
       </c>
       <c r="I181" s="9">
@@ -10155,7 +10168,7 @@
       <c r="G182" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="H182" s="4">
+      <c r="H182" s="22">
         <v>46003</v>
       </c>
       <c r="I182" s="9">
@@ -10187,7 +10200,7 @@
       <c r="G183" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="H183" s="4">
+      <c r="H183" s="22">
         <v>46003</v>
       </c>
       <c r="I183" s="9">
@@ -10219,7 +10232,7 @@
       <c r="G184" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="H184" s="4">
+      <c r="H184" s="22">
         <v>46003</v>
       </c>
       <c r="I184" s="9">
@@ -10251,7 +10264,7 @@
       <c r="G185" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="H185" s="4">
+      <c r="H185" s="22">
         <v>46003</v>
       </c>
       <c r="I185" s="9">
@@ -10283,7 +10296,7 @@
       <c r="G186" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="H186" s="4">
+      <c r="H186" s="22">
         <v>46003</v>
       </c>
       <c r="I186" s="9" t="s">
@@ -10315,7 +10328,7 @@
       <c r="G187" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H187" s="4">
+      <c r="H187" s="22">
         <v>46000</v>
       </c>
       <c r="I187" s="9" t="s">
@@ -10347,7 +10360,7 @@
       <c r="G188" s="6" t="s">
         <v>399</v>
       </c>
-      <c r="H188" s="4">
+      <c r="H188" s="22">
         <v>46000</v>
       </c>
       <c r="I188" s="9" t="s">
@@ -10379,7 +10392,7 @@
       <c r="G189" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="H189" s="4">
+      <c r="H189" s="22">
         <v>46000</v>
       </c>
       <c r="I189" s="9" t="s">
@@ -10411,7 +10424,7 @@
       <c r="G190" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="H190" s="4">
+      <c r="H190" s="22">
         <v>46000</v>
       </c>
       <c r="I190" s="9" t="s">
@@ -10443,7 +10456,7 @@
       <c r="G191" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="H191" s="4">
+      <c r="H191" s="22">
         <v>46003</v>
       </c>
       <c r="I191" s="9" t="s">
@@ -10475,7 +10488,7 @@
       <c r="G192" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="H192" s="4">
+      <c r="H192" s="22">
         <v>46000</v>
       </c>
       <c r="I192" s="9" t="s">
@@ -10507,7 +10520,7 @@
       <c r="G193" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="H193" s="4">
+      <c r="H193" s="22">
         <v>46003</v>
       </c>
       <c r="I193" s="9" t="s">
@@ -10539,7 +10552,7 @@
       <c r="G194" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="H194" s="4">
+      <c r="H194" s="22">
         <v>46000</v>
       </c>
       <c r="I194" s="9" t="s">
@@ -10571,7 +10584,7 @@
       <c r="G195" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="H195" s="4">
+      <c r="H195" s="22">
         <v>46000</v>
       </c>
       <c r="I195" s="9">
@@ -10603,7 +10616,7 @@
       <c r="G196" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="H196" s="4">
+      <c r="H196" s="22">
         <v>46000</v>
       </c>
       <c r="I196" s="9">
@@ -10635,7 +10648,7 @@
       <c r="G197" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="H197" s="4">
+      <c r="H197" s="22">
         <v>46000</v>
       </c>
       <c r="I197" s="9" t="s">
@@ -10667,7 +10680,7 @@
       <c r="G198" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="H198" s="4">
+      <c r="H198" s="22">
         <v>46000</v>
       </c>
       <c r="I198" s="9">
@@ -10699,7 +10712,7 @@
       <c r="G199" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="H199" s="5">
+      <c r="H199" s="23">
         <v>46001</v>
       </c>
       <c r="I199" s="9">
@@ -10731,7 +10744,7 @@
       <c r="G200" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="H200" s="5">
+      <c r="H200" s="23">
         <v>46001</v>
       </c>
       <c r="I200" s="9">
@@ -10763,7 +10776,7 @@
       <c r="G201" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="H201" s="5">
+      <c r="H201" s="23">
         <v>46001</v>
       </c>
       <c r="I201" s="9" t="s">
@@ -10795,7 +10808,7 @@
       <c r="G202" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="H202" s="4">
+      <c r="H202" s="22">
         <v>46008</v>
       </c>
       <c r="I202" s="9" t="s">
@@ -10827,7 +10840,7 @@
       <c r="G203" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="H203" s="5">
+      <c r="H203" s="23">
         <v>46001</v>
       </c>
       <c r="I203" s="9" t="s">
@@ -10859,7 +10872,7 @@
       <c r="G204" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="H204" s="4">
+      <c r="H204" s="22">
         <v>46008</v>
       </c>
       <c r="I204" s="9" t="s">
@@ -10891,7 +10904,7 @@
       <c r="G205" s="6" t="s">
         <v>410</v>
       </c>
-      <c r="H205" s="5">
+      <c r="H205" s="23">
         <v>46001</v>
       </c>
       <c r="I205" s="9" t="s">
@@ -10923,7 +10936,7 @@
       <c r="G206" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="H206" s="5">
+      <c r="H206" s="23">
         <v>46001</v>
       </c>
       <c r="I206" s="9" t="s">
@@ -10955,7 +10968,7 @@
       <c r="G207" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="H207" s="5">
+      <c r="H207" s="23">
         <v>46001</v>
       </c>
       <c r="I207" s="9" t="s">
@@ -10987,7 +11000,7 @@
       <c r="G208" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="H208" s="5">
+      <c r="H208" s="23">
         <v>46001</v>
       </c>
       <c r="I208" s="9" t="s">
@@ -11019,7 +11032,7 @@
       <c r="G209" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="H209" s="5">
+      <c r="H209" s="23">
         <v>46001</v>
       </c>
       <c r="I209" s="9" t="s">
@@ -11051,7 +11064,7 @@
       <c r="G210" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="H210" s="5">
+      <c r="H210" s="23">
         <v>46001</v>
       </c>
       <c r="I210" s="9" t="s">
@@ -11083,7 +11096,7 @@
       <c r="G211" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="H211" s="5">
+      <c r="H211" s="23">
         <v>46001</v>
       </c>
       <c r="I211" s="9" t="s">
@@ -11115,7 +11128,7 @@
       <c r="G212" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="H212" s="5">
+      <c r="H212" s="23">
         <v>46001</v>
       </c>
       <c r="I212" s="9" t="s">
@@ -11147,7 +11160,7 @@
       <c r="G213" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="H213" s="5">
+      <c r="H213" s="23">
         <v>46001</v>
       </c>
       <c r="I213" s="9" t="s">
@@ -11179,7 +11192,7 @@
       <c r="G214" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="H214" s="5">
+      <c r="H214" s="23">
         <v>46001</v>
       </c>
       <c r="I214" s="9" t="s">
@@ -11211,7 +11224,7 @@
       <c r="G215" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="H215" s="4">
+      <c r="H215" s="22">
         <v>46008</v>
       </c>
       <c r="I215" s="9" t="s">
@@ -11243,7 +11256,7 @@
       <c r="G216" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="H216" s="5">
+      <c r="H216" s="23">
         <v>46097</v>
       </c>
       <c r="I216" s="9" t="s">
@@ -11275,7 +11288,7 @@
       <c r="G217" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="H217" s="5">
+      <c r="H217" s="23">
         <v>46097</v>
       </c>
       <c r="I217" s="9" t="s">
@@ -11307,7 +11320,7 @@
       <c r="G218" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="H218" s="4">
+      <c r="H218" s="22">
         <v>46004</v>
       </c>
       <c r="I218" s="9" t="s">
@@ -11339,7 +11352,7 @@
       <c r="G219" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="H219" s="4">
+      <c r="H219" s="22">
         <v>46004</v>
       </c>
       <c r="I219" s="9" t="s">
@@ -11371,7 +11384,7 @@
       <c r="G220" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="H220" s="4">
+      <c r="H220" s="22">
         <v>46004</v>
       </c>
       <c r="I220" s="9" t="s">
@@ -11403,7 +11416,7 @@
       <c r="G221" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="H221" s="4">
+      <c r="H221" s="22">
         <v>46004</v>
       </c>
       <c r="I221" s="9" t="s">
@@ -11435,7 +11448,7 @@
       <c r="G222" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="H222" s="4">
+      <c r="H222" s="22">
         <v>46004</v>
       </c>
       <c r="I222" s="9" t="s">
@@ -11467,7 +11480,7 @@
       <c r="G223" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="H223" s="4">
+      <c r="H223" s="22">
         <v>46004</v>
       </c>
       <c r="I223" s="9" t="s">
@@ -11499,7 +11512,7 @@
       <c r="G224" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="H224" s="4">
+      <c r="H224" s="22">
         <v>46004</v>
       </c>
       <c r="I224" s="9" t="s">
@@ -11531,7 +11544,7 @@
       <c r="G225" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="H225" s="4">
+      <c r="H225" s="22">
         <v>46004</v>
       </c>
       <c r="I225" s="9" t="s">
@@ -11563,7 +11576,7 @@
       <c r="G226" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="H226" s="4">
+      <c r="H226" s="22">
         <v>46004</v>
       </c>
       <c r="I226" s="9" t="s">
@@ -11595,7 +11608,7 @@
       <c r="G227" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="H227" s="4">
+      <c r="H227" s="22">
         <v>46004</v>
       </c>
       <c r="I227" s="9" t="s">
@@ -11627,7 +11640,7 @@
       <c r="G228" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="H228" s="4">
+      <c r="H228" s="22">
         <v>46004</v>
       </c>
       <c r="I228" s="9" t="s">
@@ -11659,7 +11672,7 @@
       <c r="G229" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="H229" s="4">
+      <c r="H229" s="22">
         <v>46004</v>
       </c>
       <c r="I229" s="9" t="s">
@@ -11691,7 +11704,7 @@
       <c r="G230" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="H230" s="4">
+      <c r="H230" s="22">
         <v>46004</v>
       </c>
       <c r="I230" s="9" t="s">
@@ -11723,7 +11736,7 @@
       <c r="G231" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="H231" s="5">
+      <c r="H231" s="23">
         <v>46093</v>
       </c>
       <c r="I231" s="9" t="s">
@@ -11755,7 +11768,7 @@
       <c r="G232" s="6" t="s">
         <v>745</v>
       </c>
-      <c r="H232" s="5">
+      <c r="H232" s="23">
         <v>46093</v>
       </c>
       <c r="I232" s="9" t="s">
@@ -11787,7 +11800,7 @@
       <c r="G233" s="6" t="s">
         <v>746</v>
       </c>
-      <c r="H233" s="5">
+      <c r="H233" s="23">
         <v>46093</v>
       </c>
       <c r="I233" s="9" t="s">
@@ -11819,7 +11832,7 @@
       <c r="G234" s="6" t="s">
         <v>747</v>
       </c>
-      <c r="H234" s="5">
+      <c r="H234" s="23">
         <v>46094</v>
       </c>
       <c r="I234" s="9" t="s">
@@ -11851,7 +11864,7 @@
       <c r="G235" s="6" t="s">
         <v>743</v>
       </c>
-      <c r="H235" s="5">
+      <c r="H235" s="23">
         <v>46094</v>
       </c>
       <c r="I235" s="9" t="s">
@@ -11883,7 +11896,7 @@
       <c r="G236" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="H236" s="5">
+      <c r="H236" s="23">
         <v>46094</v>
       </c>
       <c r="I236" s="9" t="s">
@@ -11915,7 +11928,7 @@
       <c r="G237" s="6" t="s">
         <v>718</v>
       </c>
-      <c r="H237" s="5">
+      <c r="H237" s="23">
         <v>46099</v>
       </c>
       <c r="I237" s="9" t="s">
@@ -11947,7 +11960,7 @@
       <c r="G238" s="6" t="s">
         <v>749</v>
       </c>
-      <c r="H238" s="5">
+      <c r="H238" s="23">
         <v>46099</v>
       </c>
       <c r="I238" s="9" t="s">
@@ -11979,7 +11992,7 @@
       <c r="G239" s="6" t="s">
         <v>750</v>
       </c>
-      <c r="H239" s="5">
+      <c r="H239" s="23">
         <v>46099</v>
       </c>
       <c r="I239" s="9" t="s">
@@ -12011,7 +12024,7 @@
       <c r="G240" s="6" t="s">
         <v>695</v>
       </c>
-      <c r="H240" s="5">
+      <c r="H240" s="23">
         <v>46094</v>
       </c>
       <c r="I240" s="9" t="s">
@@ -12043,7 +12056,7 @@
       <c r="G241" s="6" t="s">
         <v>696</v>
       </c>
-      <c r="H241" s="5">
+      <c r="H241" s="23">
         <v>46094</v>
       </c>
       <c r="I241" s="9" t="s">
@@ -12075,7 +12088,7 @@
       <c r="G242" s="6" t="s">
         <v>714</v>
       </c>
-      <c r="H242" s="5">
+      <c r="H242" s="23">
         <v>46094</v>
       </c>
       <c r="I242" s="9" t="s">
@@ -12107,7 +12120,7 @@
       <c r="G243" s="6" t="s">
         <v>713</v>
       </c>
-      <c r="H243" s="5">
+      <c r="H243" s="23">
         <v>46094</v>
       </c>
       <c r="I243" s="9" t="s">
@@ -12139,7 +12152,7 @@
       <c r="G244" s="6" t="s">
         <v>712</v>
       </c>
-      <c r="H244" s="5">
+      <c r="H244" s="23">
         <v>46094</v>
       </c>
       <c r="I244" s="9" t="s">
@@ -12171,7 +12184,7 @@
       <c r="G245" s="6" t="s">
         <v>711</v>
       </c>
-      <c r="H245" s="5">
+      <c r="H245" s="23">
         <v>46094</v>
       </c>
       <c r="I245" s="9" t="s">
@@ -12203,7 +12216,7 @@
       <c r="G246" s="6" t="s">
         <v>715</v>
       </c>
-      <c r="H246" s="5">
+      <c r="H246" s="23">
         <v>46094</v>
       </c>
       <c r="I246" s="9" t="s">
@@ -12235,7 +12248,7 @@
       <c r="G247" s="6" t="s">
         <v>700</v>
       </c>
-      <c r="H247" s="5">
+      <c r="H247" s="23">
         <v>46094</v>
       </c>
       <c r="I247" s="9" t="s">
@@ -12267,7 +12280,7 @@
       <c r="G248" s="6" t="s">
         <v>701</v>
       </c>
-      <c r="H248" s="5">
+      <c r="H248" s="23">
         <v>46094</v>
       </c>
       <c r="I248" s="9" t="s">
@@ -12299,7 +12312,7 @@
       <c r="G249" s="6" t="s">
         <v>702</v>
       </c>
-      <c r="H249" s="5">
+      <c r="H249" s="23">
         <v>46094</v>
       </c>
       <c r="I249" s="9" t="s">
@@ -12331,7 +12344,7 @@
       <c r="G250" s="6" t="s">
         <v>698</v>
       </c>
-      <c r="H250" s="5">
+      <c r="H250" s="23">
         <v>46094</v>
       </c>
       <c r="I250" s="9" t="s">
@@ -12363,7 +12376,7 @@
       <c r="G251" s="6" t="s">
         <v>708</v>
       </c>
-      <c r="H251" s="5">
+      <c r="H251" s="23">
         <v>46094</v>
       </c>
       <c r="I251" s="9" t="s">
@@ -12395,7 +12408,7 @@
       <c r="G252" s="6" t="s">
         <v>719</v>
       </c>
-      <c r="H252" s="5">
+      <c r="H252" s="23">
         <v>46094</v>
       </c>
       <c r="I252" s="9" t="s">
@@ -12427,7 +12440,7 @@
       <c r="G253" s="6" t="s">
         <v>706</v>
       </c>
-      <c r="H253" s="5">
+      <c r="H253" s="23">
         <v>46094</v>
       </c>
       <c r="I253" s="9" t="s">
@@ -12459,7 +12472,7 @@
       <c r="G254" s="6" t="s">
         <v>705</v>
       </c>
-      <c r="H254" s="5">
+      <c r="H254" s="23">
         <v>46094</v>
       </c>
       <c r="I254" s="9" t="s">
@@ -12491,7 +12504,7 @@
       <c r="G255" s="6" t="s">
         <v>704</v>
       </c>
-      <c r="H255" s="5">
+      <c r="H255" s="23">
         <v>46094</v>
       </c>
       <c r="I255" s="9" t="s">
@@ -12523,7 +12536,7 @@
       <c r="G256" s="6" t="s">
         <v>703</v>
       </c>
-      <c r="H256" s="5">
+      <c r="H256" s="23">
         <v>46094</v>
       </c>
       <c r="I256" s="9" t="s">
@@ -12555,7 +12568,7 @@
       <c r="G257" s="6" t="s">
         <v>709</v>
       </c>
-      <c r="H257" s="5">
+      <c r="H257" s="23">
         <v>46094</v>
       </c>
       <c r="I257" s="9" t="s">
@@ -12587,7 +12600,7 @@
       <c r="G258" s="6" t="s">
         <v>716</v>
       </c>
-      <c r="H258" s="5">
+      <c r="H258" s="23">
         <v>46094</v>
       </c>
       <c r="I258" s="9" t="s">
@@ -12619,7 +12632,7 @@
       <c r="G259" s="6" t="s">
         <v>699</v>
       </c>
-      <c r="H259" s="5">
+      <c r="H259" s="23">
         <v>46094</v>
       </c>
       <c r="I259" s="9" t="s">
@@ -12651,7 +12664,7 @@
       <c r="G260" s="6" t="s">
         <v>710</v>
       </c>
-      <c r="H260" s="5">
+      <c r="H260" s="23">
         <v>46094</v>
       </c>
       <c r="I260" s="9" t="s">
@@ -12683,7 +12696,7 @@
       <c r="G261" s="6" t="s">
         <v>707</v>
       </c>
-      <c r="H261" s="5">
+      <c r="H261" s="23">
         <v>46094</v>
       </c>
       <c r="I261" s="9" t="s">
@@ -12715,7 +12728,7 @@
       <c r="G262" s="6" t="s">
         <v>697</v>
       </c>
-      <c r="H262" s="5">
+      <c r="H262" s="23">
         <v>46094</v>
       </c>
       <c r="I262" s="9" t="s">
@@ -12747,7 +12760,7 @@
       <c r="G263" s="6" t="s">
         <v>717</v>
       </c>
-      <c r="H263" s="5">
+      <c r="H263" s="23">
         <v>46094</v>
       </c>
       <c r="I263" s="9" t="s">
@@ -12779,7 +12792,7 @@
       <c r="G264" s="6" t="s">
         <v>731</v>
       </c>
-      <c r="H264" s="5">
+      <c r="H264" s="23">
         <v>46093</v>
       </c>
       <c r="I264" s="9" t="s">
@@ -12811,7 +12824,7 @@
       <c r="G265" s="6" t="s">
         <v>732</v>
       </c>
-      <c r="H265" s="5">
+      <c r="H265" s="23">
         <v>46093</v>
       </c>
       <c r="I265" s="9" t="s">
@@ -12843,7 +12856,7 @@
       <c r="G266" s="6" t="s">
         <v>733</v>
       </c>
-      <c r="H266" s="5">
+      <c r="H266" s="23">
         <v>46093</v>
       </c>
       <c r="I266" s="9" t="s">
@@ -12875,7 +12888,7 @@
       <c r="G267" s="6" t="s">
         <v>728</v>
       </c>
-      <c r="H267" s="5">
+      <c r="H267" s="23">
         <v>46093</v>
       </c>
       <c r="I267" s="9" t="s">
@@ -12907,7 +12920,7 @@
       <c r="G268" s="6" t="s">
         <v>729</v>
       </c>
-      <c r="H268" s="5">
+      <c r="H268" s="23">
         <v>46093</v>
       </c>
       <c r="I268" s="9" t="s">
@@ -12939,7 +12952,7 @@
       <c r="G269" s="6" t="s">
         <v>730</v>
       </c>
-      <c r="H269" s="5">
+      <c r="H269" s="23">
         <v>46093</v>
       </c>
       <c r="I269" s="9" t="s">
@@ -12971,7 +12984,7 @@
       <c r="G270" s="6" t="s">
         <v>735</v>
       </c>
-      <c r="H270" s="5">
+      <c r="H270" s="23">
         <v>46093</v>
       </c>
       <c r="I270" s="9" t="s">
@@ -13003,7 +13016,7 @@
       <c r="G271" s="6" t="s">
         <v>737</v>
       </c>
-      <c r="H271" s="5">
+      <c r="H271" s="23">
         <v>46093</v>
       </c>
       <c r="I271" s="9" t="s">
@@ -13035,7 +13048,7 @@
       <c r="G272" s="6" t="s">
         <v>736</v>
       </c>
-      <c r="H272" s="5">
+      <c r="H272" s="23">
         <v>46093</v>
       </c>
       <c r="I272" s="9" t="s">
@@ -13067,7 +13080,7 @@
       <c r="G273" s="6" t="s">
         <v>738</v>
       </c>
-      <c r="H273" s="5">
+      <c r="H273" s="23">
         <v>46093</v>
       </c>
       <c r="I273" s="9" t="s">
@@ -13099,7 +13112,7 @@
       <c r="G274" s="6" t="s">
         <v>742</v>
       </c>
-      <c r="H274" s="5">
+      <c r="H274" s="23">
         <v>46093</v>
       </c>
       <c r="I274" s="9" t="s">
@@ -13131,7 +13144,7 @@
       <c r="G275" s="6" t="s">
         <v>740</v>
       </c>
-      <c r="H275" s="5">
+      <c r="H275" s="23">
         <v>46093</v>
       </c>
       <c r="I275" s="9" t="s">
@@ -13163,7 +13176,7 @@
       <c r="G276" s="6" t="s">
         <v>734</v>
       </c>
-      <c r="H276" s="5">
+      <c r="H276" s="23">
         <v>46093</v>
       </c>
       <c r="I276" s="9" t="s">
@@ -13195,7 +13208,7 @@
       <c r="G277" s="6" t="s">
         <v>722</v>
       </c>
-      <c r="H277" s="5">
+      <c r="H277" s="23">
         <v>46095</v>
       </c>
       <c r="I277" s="9" t="s">
@@ -13227,7 +13240,7 @@
       <c r="G278" s="6" t="s">
         <v>721</v>
       </c>
-      <c r="H278" s="5">
+      <c r="H278" s="23">
         <v>46095</v>
       </c>
       <c r="I278" s="9" t="s">
@@ -13259,7 +13272,7 @@
       <c r="G279" s="6" t="s">
         <v>720</v>
       </c>
-      <c r="H279" s="5">
+      <c r="H279" s="23">
         <v>46095</v>
       </c>
       <c r="I279" s="9" t="s">
@@ -13291,7 +13304,7 @@
       <c r="G280" s="6" t="s">
         <v>726</v>
       </c>
-      <c r="H280" s="5">
+      <c r="H280" s="23">
         <v>46095</v>
       </c>
       <c r="I280" s="9" t="s">
@@ -13323,7 +13336,7 @@
       <c r="G281" s="6" t="s">
         <v>725</v>
       </c>
-      <c r="H281" s="5">
+      <c r="H281" s="23">
         <v>46095</v>
       </c>
       <c r="I281" s="9" t="s">
@@ -13355,7 +13368,7 @@
       <c r="G282" s="6" t="s">
         <v>724</v>
       </c>
-      <c r="H282" s="5">
+      <c r="H282" s="23">
         <v>46095</v>
       </c>
       <c r="I282" s="9" t="s">
@@ -13387,7 +13400,7 @@
       <c r="G283" s="6" t="s">
         <v>723</v>
       </c>
-      <c r="H283" s="5">
+      <c r="H283" s="23">
         <v>46095</v>
       </c>
       <c r="I283" s="9" t="s">
@@ -13419,7 +13432,7 @@
       <c r="G284" s="6" t="s">
         <v>741</v>
       </c>
-      <c r="H284" s="5">
+      <c r="H284" s="23">
         <v>46095</v>
       </c>
       <c r="I284" s="9" t="s">
@@ -13451,7 +13464,7 @@
       <c r="G285" s="6" t="s">
         <v>739</v>
       </c>
-      <c r="H285" s="5">
+      <c r="H285" s="23">
         <v>46095</v>
       </c>
       <c r="I285" s="9" t="s">
@@ -13483,7 +13496,7 @@
       <c r="G286" s="6" t="s">
         <v>727</v>
       </c>
-      <c r="H286" s="5">
+      <c r="H286" s="23">
         <v>46095</v>
       </c>
       <c r="I286" s="9" t="s">
@@ -13515,7 +13528,7 @@
       <c r="G287" s="6" t="s">
         <v>937</v>
       </c>
-      <c r="H287" s="5">
+      <c r="H287" s="23">
         <v>46095</v>
       </c>
       <c r="I287" s="9" t="s">
@@ -13545,7 +13558,7 @@
       <c r="G288" s="12" t="s">
         <v>923</v>
       </c>
-      <c r="H288" s="14">
+      <c r="H288" s="24">
         <v>46100</v>
       </c>
       <c r="I288" s="9" t="s">
@@ -13575,7 +13588,7 @@
       <c r="G289" s="12" t="s">
         <v>923</v>
       </c>
-      <c r="H289" s="14">
+      <c r="H289" s="24">
         <v>46100</v>
       </c>
       <c r="I289" s="9" t="s">
@@ -13605,7 +13618,7 @@
       <c r="G290" s="12" t="s">
         <v>923</v>
       </c>
-      <c r="H290" s="14">
+      <c r="H290" s="24">
         <v>46100</v>
       </c>
       <c r="I290" s="9" t="s">
@@ -13635,7 +13648,7 @@
       <c r="G291" s="8" t="s">
         <v>924</v>
       </c>
-      <c r="H291" s="5">
+      <c r="H291" s="23">
         <v>46100</v>
       </c>
       <c r="I291" s="9" t="s">
@@ -13665,7 +13678,7 @@
       <c r="G292" s="8" t="s">
         <v>925</v>
       </c>
-      <c r="H292" s="5">
+      <c r="H292" s="23">
         <v>46100</v>
       </c>
       <c r="I292" s="9" t="s">
@@ -13695,7 +13708,7 @@
       <c r="G293" s="12" t="s">
         <v>926</v>
       </c>
-      <c r="H293" s="14">
+      <c r="H293" s="24">
         <v>46100</v>
       </c>
       <c r="I293" s="9" t="s">
@@ -13725,7 +13738,7 @@
       <c r="G294" s="12" t="s">
         <v>926</v>
       </c>
-      <c r="H294" s="14">
+      <c r="H294" s="24">
         <v>46100</v>
       </c>
       <c r="I294" s="9" t="s">
@@ -13755,7 +13768,7 @@
       <c r="G295" s="12" t="s">
         <v>926</v>
       </c>
-      <c r="H295" s="14">
+      <c r="H295" s="24">
         <v>46100</v>
       </c>
       <c r="I295" s="9" t="s">
@@ -13785,7 +13798,7 @@
       <c r="G296" s="12" t="s">
         <v>927</v>
       </c>
-      <c r="H296" s="14">
+      <c r="H296" s="24">
         <v>46106</v>
       </c>
       <c r="I296" s="9" t="s">
@@ -13815,7 +13828,7 @@
       <c r="G297" s="12" t="s">
         <v>927</v>
       </c>
-      <c r="H297" s="14">
+      <c r="H297" s="24">
         <v>46106</v>
       </c>
       <c r="I297" s="9" t="s">
@@ -13845,7 +13858,7 @@
       <c r="G298" s="8" t="s">
         <v>928</v>
       </c>
-      <c r="H298" s="5">
+      <c r="H298" s="23">
         <v>46106</v>
       </c>
       <c r="I298" s="9" t="s">
@@ -13875,7 +13888,7 @@
       <c r="G299" s="8" t="s">
         <v>929</v>
       </c>
-      <c r="H299" s="5">
+      <c r="H299" s="23">
         <v>46106</v>
       </c>
       <c r="I299" s="9" t="s">
@@ -13905,7 +13918,7 @@
       <c r="G300" s="8" t="s">
         <v>775</v>
       </c>
-      <c r="H300" s="5">
+      <c r="H300" s="23">
         <v>46106</v>
       </c>
       <c r="I300" s="9" t="s">
@@ -13935,7 +13948,7 @@
       <c r="G301" s="8" t="s">
         <v>775</v>
       </c>
-      <c r="H301" s="5">
+      <c r="H301" s="23">
         <v>46106</v>
       </c>
       <c r="I301" s="9" t="s">
@@ -13965,7 +13978,7 @@
       <c r="G302" s="12" t="s">
         <v>930</v>
       </c>
-      <c r="H302" s="14">
+      <c r="H302" s="24">
         <v>46106</v>
       </c>
       <c r="I302" s="9" t="s">
@@ -13995,7 +14008,7 @@
       <c r="G303" s="12" t="s">
         <v>930</v>
       </c>
-      <c r="H303" s="14">
+      <c r="H303" s="24">
         <v>46106</v>
       </c>
       <c r="I303" s="9" t="s">
@@ -14025,7 +14038,7 @@
       <c r="G304" s="12" t="s">
         <v>931</v>
       </c>
-      <c r="H304" s="14">
+      <c r="H304" s="24">
         <v>46112</v>
       </c>
       <c r="I304" s="9" t="s">
@@ -14055,7 +14068,7 @@
       <c r="G305" s="12" t="s">
         <v>931</v>
       </c>
-      <c r="H305" s="14">
+      <c r="H305" s="24">
         <v>46112</v>
       </c>
       <c r="I305" s="9" t="s">
@@ -14085,7 +14098,7 @@
       <c r="G306" s="8" t="s">
         <v>932</v>
       </c>
-      <c r="H306" s="5">
+      <c r="H306" s="23">
         <v>46100</v>
       </c>
       <c r="I306" s="9" t="s">
@@ -14115,7 +14128,7 @@
       <c r="G307" s="12" t="s">
         <v>933</v>
       </c>
-      <c r="H307" s="14">
+      <c r="H307" s="24">
         <v>46100</v>
       </c>
       <c r="I307" s="9" t="s">
@@ -14145,7 +14158,7 @@
       <c r="G308" s="12" t="s">
         <v>933</v>
       </c>
-      <c r="H308" s="14">
+      <c r="H308" s="24">
         <v>46100</v>
       </c>
       <c r="I308" s="9" t="s">
@@ -14175,7 +14188,7 @@
       <c r="G309" s="12" t="s">
         <v>934</v>
       </c>
-      <c r="H309" s="14">
+      <c r="H309" s="24">
         <v>46100</v>
       </c>
       <c r="I309" s="9" t="s">
@@ -14205,7 +14218,7 @@
       <c r="G310" s="8" t="s">
         <v>935</v>
       </c>
-      <c r="H310" s="5">
+      <c r="H310" s="23">
         <v>46100</v>
       </c>
       <c r="I310" s="9" t="s">
@@ -14233,7 +14246,7 @@
       </c>
       <c r="F311" s="2"/>
       <c r="G311" s="6"/>
-      <c r="H311" s="6"/>
+      <c r="H311" s="25"/>
       <c r="I311" s="6"/>
       <c r="J311" s="6"/>
     </row>
@@ -14255,7 +14268,7 @@
       </c>
       <c r="F312" s="2"/>
       <c r="G312" s="6"/>
-      <c r="H312" s="6"/>
+      <c r="H312" s="25"/>
       <c r="I312" s="6"/>
       <c r="J312" s="6"/>
     </row>
@@ -14277,7 +14290,7 @@
       </c>
       <c r="F313" s="2"/>
       <c r="G313" s="6"/>
-      <c r="H313" s="6"/>
+      <c r="H313" s="25"/>
       <c r="I313" s="6"/>
       <c r="J313" s="6"/>
     </row>
@@ -14299,7 +14312,7 @@
       </c>
       <c r="F314" s="2"/>
       <c r="G314" s="6"/>
-      <c r="H314" s="6"/>
+      <c r="H314" s="25"/>
       <c r="I314" s="6"/>
       <c r="J314" s="6"/>
     </row>
@@ -14321,7 +14334,7 @@
       </c>
       <c r="F315" s="2"/>
       <c r="G315" s="6"/>
-      <c r="H315" s="6"/>
+      <c r="H315" s="25"/>
       <c r="I315" s="6"/>
       <c r="J315" s="6"/>
     </row>
@@ -14343,7 +14356,7 @@
       </c>
       <c r="F316" s="2"/>
       <c r="G316" s="6"/>
-      <c r="H316" s="6"/>
+      <c r="H316" s="25"/>
       <c r="I316" s="6"/>
       <c r="J316" s="6"/>
     </row>
@@ -14365,7 +14378,7 @@
       </c>
       <c r="F317" s="2"/>
       <c r="G317" s="6"/>
-      <c r="H317" s="6"/>
+      <c r="H317" s="25"/>
       <c r="I317" s="6"/>
       <c r="J317" s="6"/>
     </row>
@@ -14387,7 +14400,7 @@
       </c>
       <c r="F318" s="2"/>
       <c r="G318" s="6"/>
-      <c r="H318" s="6"/>
+      <c r="H318" s="25"/>
       <c r="I318" s="6"/>
       <c r="J318" s="6"/>
     </row>
@@ -14409,7 +14422,7 @@
       </c>
       <c r="F319" s="2"/>
       <c r="G319" s="6"/>
-      <c r="H319" s="6"/>
+      <c r="H319" s="25"/>
       <c r="I319" s="6"/>
       <c r="J319" s="6"/>
     </row>
@@ -14431,7 +14444,7 @@
       </c>
       <c r="F320" s="2"/>
       <c r="G320" s="6"/>
-      <c r="H320" s="6"/>
+      <c r="H320" s="25"/>
       <c r="I320" s="6"/>
       <c r="J320" s="6"/>
     </row>
@@ -14453,7 +14466,7 @@
       </c>
       <c r="F321" s="2"/>
       <c r="G321" s="6"/>
-      <c r="H321" s="6"/>
+      <c r="H321" s="25"/>
       <c r="I321" s="6"/>
       <c r="J321" s="6"/>
     </row>
@@ -14475,7 +14488,7 @@
       </c>
       <c r="F322" s="2"/>
       <c r="G322" s="6"/>
-      <c r="H322" s="6"/>
+      <c r="H322" s="25"/>
       <c r="I322" s="6"/>
       <c r="J322" s="6"/>
     </row>
@@ -14497,7 +14510,7 @@
       </c>
       <c r="F323" s="7"/>
       <c r="G323" s="6"/>
-      <c r="H323" s="6"/>
+      <c r="H323" s="25"/>
       <c r="I323" s="6"/>
       <c r="J323" s="6"/>
     </row>
@@ -14519,7 +14532,7 @@
       </c>
       <c r="F324" s="7"/>
       <c r="G324" s="6"/>
-      <c r="H324" s="6"/>
+      <c r="H324" s="25"/>
       <c r="I324" s="6"/>
       <c r="J324" s="6"/>
     </row>
@@ -14541,7 +14554,7 @@
       </c>
       <c r="F325" s="7"/>
       <c r="G325" s="6"/>
-      <c r="H325" s="6"/>
+      <c r="H325" s="25"/>
       <c r="I325" s="6"/>
       <c r="J325" s="6"/>
     </row>
@@ -14563,7 +14576,7 @@
       </c>
       <c r="F326" s="7"/>
       <c r="G326" s="6"/>
-      <c r="H326" s="6"/>
+      <c r="H326" s="25"/>
       <c r="I326" s="6"/>
       <c r="J326" s="6"/>
     </row>
@@ -14585,7 +14598,7 @@
       </c>
       <c r="F327" s="2"/>
       <c r="G327" s="6"/>
-      <c r="H327" s="6"/>
+      <c r="H327" s="25"/>
       <c r="I327" s="6"/>
       <c r="J327" s="6"/>
     </row>
@@ -14607,7 +14620,7 @@
       </c>
       <c r="F328" s="7"/>
       <c r="G328" s="6"/>
-      <c r="H328" s="6"/>
+      <c r="H328" s="25"/>
       <c r="I328" s="6"/>
       <c r="J328" s="6"/>
     </row>
@@ -14629,7 +14642,7 @@
       </c>
       <c r="F329" s="7"/>
       <c r="G329" s="6"/>
-      <c r="H329" s="6"/>
+      <c r="H329" s="25"/>
       <c r="I329" s="6"/>
       <c r="J329" s="6"/>
     </row>
@@ -14651,7 +14664,7 @@
       </c>
       <c r="F330" s="7"/>
       <c r="G330" s="6"/>
-      <c r="H330" s="6"/>
+      <c r="H330" s="25"/>
       <c r="I330" s="6"/>
       <c r="J330" s="6"/>
     </row>
@@ -14673,7 +14686,7 @@
       </c>
       <c r="F331" s="7"/>
       <c r="G331" s="6"/>
-      <c r="H331" s="6"/>
+      <c r="H331" s="25"/>
       <c r="I331" s="6"/>
       <c r="J331" s="6"/>
     </row>
@@ -14695,7 +14708,7 @@
       </c>
       <c r="F332" s="7"/>
       <c r="G332" s="6"/>
-      <c r="H332" s="6"/>
+      <c r="H332" s="25"/>
       <c r="I332" s="6"/>
       <c r="J332" s="6"/>
     </row>
@@ -14717,7 +14730,7 @@
       </c>
       <c r="F333" s="7"/>
       <c r="G333" s="6"/>
-      <c r="H333" s="6"/>
+      <c r="H333" s="25"/>
       <c r="I333" s="6"/>
       <c r="J333" s="6"/>
     </row>
@@ -14739,7 +14752,7 @@
       </c>
       <c r="F334" s="7"/>
       <c r="G334" s="6"/>
-      <c r="H334" s="6"/>
+      <c r="H334" s="25"/>
       <c r="I334" s="6"/>
       <c r="J334" s="6"/>
     </row>
@@ -14761,7 +14774,7 @@
       </c>
       <c r="F335" s="7"/>
       <c r="G335" s="6"/>
-      <c r="H335" s="6"/>
+      <c r="H335" s="25"/>
       <c r="I335" s="6"/>
       <c r="J335" s="6"/>
     </row>
@@ -14783,7 +14796,7 @@
       </c>
       <c r="F336" s="7"/>
       <c r="G336" s="6"/>
-      <c r="H336" s="6"/>
+      <c r="H336" s="25"/>
       <c r="I336" s="6"/>
       <c r="J336" s="6"/>
     </row>
@@ -14805,7 +14818,7 @@
       </c>
       <c r="F337" s="7"/>
       <c r="G337" s="6"/>
-      <c r="H337" s="6"/>
+      <c r="H337" s="25"/>
       <c r="I337" s="6"/>
       <c r="J337" s="6"/>
     </row>
@@ -14827,7 +14840,7 @@
       </c>
       <c r="F338" s="7"/>
       <c r="G338" s="6"/>
-      <c r="H338" s="6"/>
+      <c r="H338" s="25"/>
       <c r="I338" s="6"/>
       <c r="J338" s="6"/>
     </row>
@@ -14849,7 +14862,7 @@
       </c>
       <c r="F339" s="7"/>
       <c r="G339" s="6"/>
-      <c r="H339" s="6"/>
+      <c r="H339" s="25"/>
       <c r="I339" s="6"/>
       <c r="J339" s="6"/>
     </row>
@@ -14871,7 +14884,7 @@
       </c>
       <c r="F340" s="7"/>
       <c r="G340" s="6"/>
-      <c r="H340" s="6"/>
+      <c r="H340" s="25"/>
       <c r="I340" s="6"/>
       <c r="J340" s="6"/>
     </row>
@@ -14895,7 +14908,7 @@
       <c r="G341" s="6" t="s">
         <v>915</v>
       </c>
-      <c r="H341" s="5">
+      <c r="H341" s="23">
         <v>46099</v>
       </c>
       <c r="I341" s="9" t="s">
@@ -14925,7 +14938,7 @@
       <c r="G342" s="13" t="s">
         <v>916</v>
       </c>
-      <c r="H342" s="14">
+      <c r="H342" s="24">
         <v>46099</v>
       </c>
       <c r="I342" s="15" t="s">
@@ -14955,7 +14968,7 @@
       <c r="G343" s="13" t="s">
         <v>916</v>
       </c>
-      <c r="H343" s="14">
+      <c r="H343" s="24">
         <v>46099</v>
       </c>
       <c r="I343" s="15" t="s">
@@ -14985,7 +14998,7 @@
       <c r="G344" s="13" t="s">
         <v>917</v>
       </c>
-      <c r="H344" s="14">
+      <c r="H344" s="24">
         <v>46107</v>
       </c>
       <c r="I344" s="15" t="s">
@@ -15015,7 +15028,7 @@
       <c r="G345" s="13" t="s">
         <v>917</v>
       </c>
-      <c r="H345" s="14">
+      <c r="H345" s="24">
         <v>46107</v>
       </c>
       <c r="I345" s="15" t="s">
@@ -15045,7 +15058,7 @@
       <c r="G346" s="13" t="s">
         <v>918</v>
       </c>
-      <c r="H346" s="14">
+      <c r="H346" s="24">
         <v>46100</v>
       </c>
       <c r="I346" s="15" t="s">
@@ -15075,7 +15088,7 @@
       <c r="G347" s="13" t="s">
         <v>918</v>
       </c>
-      <c r="H347" s="14">
+      <c r="H347" s="24">
         <v>46100</v>
       </c>
       <c r="I347" s="15" t="s">
@@ -15105,7 +15118,7 @@
       <c r="G348" s="13" t="s">
         <v>919</v>
       </c>
-      <c r="H348" s="14">
+      <c r="H348" s="24">
         <v>46101</v>
       </c>
       <c r="I348" s="15" t="s">
@@ -15135,7 +15148,7 @@
       <c r="G349" s="13" t="s">
         <v>919</v>
       </c>
-      <c r="H349" s="14">
+      <c r="H349" s="24">
         <v>46101</v>
       </c>
       <c r="I349" s="15" t="s">
@@ -15165,7 +15178,7 @@
       <c r="G350" s="13" t="s">
         <v>920</v>
       </c>
-      <c r="H350" s="14">
+      <c r="H350" s="24">
         <v>46101</v>
       </c>
       <c r="I350" s="15" t="s">
@@ -15195,7 +15208,7 @@
       <c r="G351" s="13" t="s">
         <v>920</v>
       </c>
-      <c r="H351" s="14">
+      <c r="H351" s="24">
         <v>46101</v>
       </c>
       <c r="I351" s="15" t="s">
@@ -15225,7 +15238,7 @@
       <c r="G352" s="6" t="s">
         <v>921</v>
       </c>
-      <c r="H352" s="5">
+      <c r="H352" s="23">
         <v>46099</v>
       </c>
       <c r="I352" s="9" t="s">
@@ -15255,7 +15268,7 @@
       <c r="G353" s="6" t="s">
         <v>922</v>
       </c>
-      <c r="H353" s="5">
+      <c r="H353" s="23">
         <v>46099</v>
       </c>
       <c r="I353" s="9" t="s">
@@ -15285,7 +15298,7 @@
       <c r="G354" s="13" t="s">
         <v>893</v>
       </c>
-      <c r="H354" s="14">
+      <c r="H354" s="24">
         <v>46097</v>
       </c>
       <c r="I354" s="15" t="s">
@@ -15315,7 +15328,7 @@
       <c r="G355" s="13" t="s">
         <v>893</v>
       </c>
-      <c r="H355" s="14">
+      <c r="H355" s="24">
         <v>46097</v>
       </c>
       <c r="I355" s="15" t="s">
@@ -15345,7 +15358,7 @@
       <c r="G356" s="13" t="s">
         <v>893</v>
       </c>
-      <c r="H356" s="14">
+      <c r="H356" s="24">
         <v>46097</v>
       </c>
       <c r="I356" s="15" t="s">
@@ -15375,7 +15388,7 @@
       <c r="G357" s="13" t="s">
         <v>894</v>
       </c>
-      <c r="H357" s="14">
+      <c r="H357" s="24">
         <v>46097</v>
       </c>
       <c r="I357" s="15" t="s">
@@ -15405,7 +15418,7 @@
       <c r="G358" s="13" t="s">
         <v>894</v>
       </c>
-      <c r="H358" s="14">
+      <c r="H358" s="24">
         <v>46097</v>
       </c>
       <c r="I358" s="15" t="s">
@@ -15435,7 +15448,7 @@
       <c r="G359" s="13" t="s">
         <v>895</v>
       </c>
-      <c r="H359" s="14">
+      <c r="H359" s="24">
         <v>46097</v>
       </c>
       <c r="I359" s="15" t="s">
@@ -15465,7 +15478,7 @@
       <c r="G360" s="13" t="s">
         <v>895</v>
       </c>
-      <c r="H360" s="14">
+      <c r="H360" s="24">
         <v>46097</v>
       </c>
       <c r="I360" s="15" t="s">
@@ -15495,7 +15508,7 @@
       <c r="G361" s="13" t="s">
         <v>895</v>
       </c>
-      <c r="H361" s="14">
+      <c r="H361" s="24">
         <v>46097</v>
       </c>
       <c r="I361" s="15" t="s">
@@ -15525,7 +15538,7 @@
       <c r="G362" s="13" t="s">
         <v>895</v>
       </c>
-      <c r="H362" s="14">
+      <c r="H362" s="24">
         <v>46097</v>
       </c>
       <c r="I362" s="15" t="s">
@@ -15555,7 +15568,7 @@
       <c r="G363" s="13" t="s">
         <v>896</v>
       </c>
-      <c r="H363" s="14">
+      <c r="H363" s="24">
         <v>46097</v>
       </c>
       <c r="I363" s="15" t="s">
@@ -15585,7 +15598,7 @@
       <c r="G364" s="13" t="s">
         <v>896</v>
       </c>
-      <c r="H364" s="14">
+      <c r="H364" s="24">
         <v>46097</v>
       </c>
       <c r="I364" s="15" t="s">
@@ -15615,7 +15628,7 @@
       <c r="G365" s="13" t="s">
         <v>896</v>
       </c>
-      <c r="H365" s="14">
+      <c r="H365" s="24">
         <v>46097</v>
       </c>
       <c r="I365" s="15" t="s">
@@ -15645,7 +15658,7 @@
       <c r="G366" s="13" t="s">
         <v>897</v>
       </c>
-      <c r="H366" s="14">
+      <c r="H366" s="24">
         <v>46099</v>
       </c>
       <c r="I366" s="15" t="s">
@@ -15675,7 +15688,7 @@
       <c r="G367" s="13" t="s">
         <v>897</v>
       </c>
-      <c r="H367" s="14">
+      <c r="H367" s="24">
         <v>46099</v>
       </c>
       <c r="I367" s="15" t="s">
@@ -15705,7 +15718,7 @@
       <c r="G368" s="13" t="s">
         <v>898</v>
       </c>
-      <c r="H368" s="14">
+      <c r="H368" s="24">
         <v>46097</v>
       </c>
       <c r="I368" s="15" t="s">
@@ -15735,7 +15748,7 @@
       <c r="G369" s="13" t="s">
         <v>898</v>
       </c>
-      <c r="H369" s="14">
+      <c r="H369" s="24">
         <v>46097</v>
       </c>
       <c r="I369" s="15" t="s">
@@ -15765,7 +15778,7 @@
       <c r="G370" s="13" t="s">
         <v>899</v>
       </c>
-      <c r="H370" s="14">
+      <c r="H370" s="24">
         <v>46107</v>
       </c>
       <c r="I370" s="15" t="s">
@@ -15795,7 +15808,7 @@
       <c r="G371" s="13" t="s">
         <v>899</v>
       </c>
-      <c r="H371" s="14">
+      <c r="H371" s="24">
         <v>46107</v>
       </c>
       <c r="I371" s="15" t="s">
@@ -15825,7 +15838,7 @@
       <c r="G372" s="13" t="s">
         <v>899</v>
       </c>
-      <c r="H372" s="14">
+      <c r="H372" s="24">
         <v>46107</v>
       </c>
       <c r="I372" s="15" t="s">
@@ -15855,7 +15868,7 @@
       <c r="G373" s="13" t="s">
         <v>899</v>
       </c>
-      <c r="H373" s="14">
+      <c r="H373" s="24">
         <v>46107</v>
       </c>
       <c r="I373" s="15" t="s">
@@ -15885,7 +15898,7 @@
       <c r="G374" s="13" t="s">
         <v>951</v>
       </c>
-      <c r="H374" s="14">
+      <c r="H374" s="24">
         <v>46107</v>
       </c>
       <c r="I374" s="15" t="s">
@@ -15915,7 +15928,7 @@
       <c r="G375" s="13" t="s">
         <v>900</v>
       </c>
-      <c r="H375" s="14">
+      <c r="H375" s="24">
         <v>46097</v>
       </c>
       <c r="I375" s="15" t="s">
@@ -15945,7 +15958,7 @@
       <c r="G376" s="13" t="s">
         <v>900</v>
       </c>
-      <c r="H376" s="14">
+      <c r="H376" s="24">
         <v>46097</v>
       </c>
       <c r="I376" s="15" t="s">
@@ -15975,7 +15988,7 @@
       <c r="G377" s="6" t="s">
         <v>901</v>
       </c>
-      <c r="H377" s="5">
+      <c r="H377" s="23">
         <v>46097</v>
       </c>
       <c r="I377" s="11" t="s">
@@ -16005,7 +16018,7 @@
       <c r="G378" s="6" t="s">
         <v>902</v>
       </c>
-      <c r="H378" s="5">
+      <c r="H378" s="23">
         <v>46098</v>
       </c>
       <c r="I378" s="11" t="s">
@@ -16035,7 +16048,7 @@
       <c r="G379" s="13" t="s">
         <v>903</v>
       </c>
-      <c r="H379" s="14">
+      <c r="H379" s="24">
         <v>46098</v>
       </c>
       <c r="I379" s="15" t="s">
@@ -16065,7 +16078,7 @@
       <c r="G380" s="13" t="s">
         <v>903</v>
       </c>
-      <c r="H380" s="14">
+      <c r="H380" s="24">
         <v>46098</v>
       </c>
       <c r="I380" s="15" t="s">
@@ -16095,7 +16108,7 @@
       <c r="G381" s="13" t="s">
         <v>904</v>
       </c>
-      <c r="H381" s="14">
+      <c r="H381" s="24">
         <v>46098</v>
       </c>
       <c r="I381" s="15" t="s">
@@ -16125,7 +16138,7 @@
       <c r="G382" s="13" t="s">
         <v>904</v>
       </c>
-      <c r="H382" s="14">
+      <c r="H382" s="24">
         <v>46098</v>
       </c>
       <c r="I382" s="15" t="s">
@@ -16155,7 +16168,7 @@
       <c r="G383" s="6" t="s">
         <v>905</v>
       </c>
-      <c r="H383" s="5">
+      <c r="H383" s="23">
         <v>46098</v>
       </c>
       <c r="I383" s="11" t="s">
@@ -16185,7 +16198,7 @@
       <c r="G384" s="6" t="s">
         <v>906</v>
       </c>
-      <c r="H384" s="5">
+      <c r="H384" s="23">
         <v>46098</v>
       </c>
       <c r="I384" s="11" t="s">
@@ -16215,7 +16228,7 @@
       <c r="G385" s="13" t="s">
         <v>907</v>
       </c>
-      <c r="H385" s="14">
+      <c r="H385" s="24">
         <v>46098</v>
       </c>
       <c r="I385" s="15" t="s">
@@ -16245,7 +16258,7 @@
       <c r="G386" s="13" t="s">
         <v>907</v>
       </c>
-      <c r="H386" s="14">
+      <c r="H386" s="24">
         <v>46098</v>
       </c>
       <c r="I386" s="15" t="s">
@@ -16275,7 +16288,7 @@
       <c r="G387" s="6" t="s">
         <v>908</v>
       </c>
-      <c r="H387" s="5">
+      <c r="H387" s="23">
         <v>46107</v>
       </c>
       <c r="I387" s="11" t="s">
@@ -16305,7 +16318,7 @@
       <c r="G388" s="6" t="s">
         <v>909</v>
       </c>
-      <c r="H388" s="5">
+      <c r="H388" s="23">
         <v>46100</v>
       </c>
       <c r="I388" s="11" t="s">
@@ -16335,7 +16348,7 @@
       <c r="G389" s="6" t="s">
         <v>910</v>
       </c>
-      <c r="H389" s="5">
+      <c r="H389" s="23">
         <v>46098</v>
       </c>
       <c r="I389" s="11" t="s">
@@ -16365,7 +16378,7 @@
       <c r="G390" s="6" t="s">
         <v>911</v>
       </c>
-      <c r="H390" s="5">
+      <c r="H390" s="23">
         <v>46098</v>
       </c>
       <c r="I390" s="11" t="s">
@@ -16395,7 +16408,7 @@
       <c r="G391" s="13" t="s">
         <v>912</v>
       </c>
-      <c r="H391" s="14">
+      <c r="H391" s="24">
         <v>46097</v>
       </c>
       <c r="I391" s="15" t="s">
@@ -16425,7 +16438,7 @@
       <c r="G392" s="13" t="s">
         <v>912</v>
       </c>
-      <c r="H392" s="14">
+      <c r="H392" s="24">
         <v>46097</v>
       </c>
       <c r="I392" s="15" t="s">
@@ -16455,7 +16468,7 @@
       <c r="G393" s="13" t="s">
         <v>912</v>
       </c>
-      <c r="H393" s="14">
+      <c r="H393" s="24">
         <v>46097</v>
       </c>
       <c r="I393" s="15" t="s">
@@ -16485,7 +16498,7 @@
       <c r="G394" s="13" t="s">
         <v>913</v>
       </c>
-      <c r="H394" s="14">
+      <c r="H394" s="24">
         <v>46098</v>
       </c>
       <c r="I394" s="15" t="s">
@@ -16515,7 +16528,7 @@
       <c r="G395" s="13" t="s">
         <v>913</v>
       </c>
-      <c r="H395" s="14">
+      <c r="H395" s="24">
         <v>46098</v>
       </c>
       <c r="I395" s="15" t="s">
@@ -16545,7 +16558,7 @@
       <c r="G396" s="13" t="s">
         <v>913</v>
       </c>
-      <c r="H396" s="14">
+      <c r="H396" s="24">
         <v>46098</v>
       </c>
       <c r="I396" s="15" t="s">
@@ -16575,7 +16588,7 @@
       <c r="G397" s="13" t="s">
         <v>913</v>
       </c>
-      <c r="H397" s="14">
+      <c r="H397" s="24">
         <v>46098</v>
       </c>
       <c r="I397" s="15" t="s">
@@ -16605,7 +16618,7 @@
       <c r="G398" s="13" t="s">
         <v>913</v>
       </c>
-      <c r="H398" s="14">
+      <c r="H398" s="24">
         <v>46098</v>
       </c>
       <c r="I398" s="15" t="s">
@@ -16635,7 +16648,7 @@
       <c r="G399" s="6" t="s">
         <v>914</v>
       </c>
-      <c r="H399" s="5">
+      <c r="H399" s="23">
         <v>46099</v>
       </c>
       <c r="I399" s="9" t="s">
@@ -16665,7 +16678,7 @@
       <c r="G400" s="6" t="s">
         <v>914</v>
       </c>
-      <c r="H400" s="5">
+      <c r="H400" s="23">
         <v>46099</v>
       </c>
       <c r="I400" s="9" t="s">
@@ -16695,7 +16708,7 @@
       <c r="G401" s="6" t="s">
         <v>914</v>
       </c>
-      <c r="H401" s="5">
+      <c r="H401" s="23">
         <v>46099</v>
       </c>
       <c r="I401" s="9" t="s">
@@ -16725,7 +16738,7 @@
       <c r="G402" s="6" t="s">
         <v>914</v>
       </c>
-      <c r="H402" s="5">
+      <c r="H402" s="23">
         <v>46099</v>
       </c>
       <c r="I402" s="9" t="s">
@@ -16736,7 +16749,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J287" xr:uid="{576B4F00-2F9D-4914-B9F2-1520968A43B1}"/>
+  <autoFilter ref="A1:J402" xr:uid="{576B4F00-2F9D-4914-B9F2-1520968A43B1}"/>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="H311:H340">
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>

</xml_diff>